<commit_message>
update scan/monitor, add schedule module, refresh scan2fetch.sql
</commit_message>
<xml_diff>
--- a/sample_students.xlsx
+++ b/sample_students.xlsx
@@ -1,21 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\scan2fetch\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C368A052-D735-4D6D-A054-0E116A9B5971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Students" sheetId="1" r:id="rId4"/>
+    <sheet name="Students" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="181">
   <si>
     <t>Student First Name</t>
   </si>
@@ -543,28 +553,35 @@
   </si>
   <si>
     <t>09171000049</t>
+  </si>
+  <si>
+    <t>jaylin</t>
+  </si>
+  <si>
+    <t>wala</t>
+  </si>
+  <si>
+    <t>lim</t>
+  </si>
+  <si>
+    <t>shana</t>
+  </si>
+  <si>
+    <t>joy</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
@@ -597,14 +614,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -894,25 +919,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:I51"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -941,7 +963,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -964,7 +986,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -987,7 +1009,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -1010,7 +1032,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -1033,7 +1055,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1056,7 +1078,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -1079,7 +1101,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -1102,7 +1124,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>52</v>
       </c>
@@ -1125,7 +1147,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>57</v>
       </c>
@@ -1148,7 +1170,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>63</v>
       </c>
@@ -1171,7 +1193,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -1194,7 +1216,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -1217,7 +1239,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>76</v>
       </c>
@@ -1240,7 +1262,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>81</v>
       </c>
@@ -1263,7 +1285,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>74</v>
       </c>
@@ -1286,7 +1308,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>88</v>
       </c>
@@ -1309,7 +1331,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>91</v>
       </c>
@@ -1332,7 +1354,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>95</v>
       </c>
@@ -1355,7 +1377,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -1378,7 +1400,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>101</v>
       </c>
@@ -1401,7 +1423,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>103</v>
       </c>
@@ -1424,7 +1446,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>84</v>
       </c>
@@ -1447,7 +1469,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>110</v>
       </c>
@@ -1470,7 +1492,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>114</v>
       </c>
@@ -1493,7 +1515,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>108</v>
       </c>
@@ -1516,7 +1538,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -1539,7 +1561,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>16</v>
       </c>
@@ -1562,7 +1584,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -1585,7 +1607,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -1608,7 +1630,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>19</v>
       </c>
@@ -1631,7 +1653,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>40</v>
       </c>
@@ -1654,7 +1676,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>46</v>
       </c>
@@ -1677,7 +1699,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>52</v>
       </c>
@@ -1700,7 +1722,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>57</v>
       </c>
@@ -1723,7 +1745,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>63</v>
       </c>
@@ -1746,7 +1768,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>67</v>
       </c>
@@ -1769,7 +1791,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>33</v>
       </c>
@@ -1792,7 +1814,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>76</v>
       </c>
@@ -1815,7 +1837,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>81</v>
       </c>
@@ -1838,7 +1860,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>74</v>
       </c>
@@ -1861,7 +1883,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>88</v>
       </c>
@@ -1884,7 +1906,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>91</v>
       </c>
@@ -1907,7 +1929,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>95</v>
       </c>
@@ -1930,7 +1952,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>43</v>
       </c>
@@ -1953,7 +1975,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>101</v>
       </c>
@@ -1976,7 +1998,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>103</v>
       </c>
@@ -1999,7 +2021,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>84</v>
       </c>
@@ -2022,7 +2044,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>110</v>
       </c>
@@ -2045,7 +2067,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="50" spans="1:9">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>114</v>
       </c>
@@ -2068,7 +2090,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:9">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>108</v>
       </c>
@@ -2091,9 +2113,33 @@
         <v>22</v>
       </c>
     </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>176</v>
+      </c>
+      <c r="B52" t="s">
+        <v>177</v>
+      </c>
+      <c r="C52" t="s">
+        <v>178</v>
+      </c>
+      <c r="D52" t="s">
+        <v>54</v>
+      </c>
+      <c r="E52" t="s">
+        <v>179</v>
+      </c>
+      <c r="G52" t="s">
+        <v>180</v>
+      </c>
+      <c r="H52">
+        <v>9995011147</v>
+      </c>
+      <c r="I52" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>